<commit_message>
Refactor engine to single input-output Excel approach and remove unused functions
</commit_message>
<xml_diff>
--- a/test-data/demo_test_data.xlsx
+++ b/test-data/demo_test_data.xlsx
@@ -3,18 +3,15 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="21000" windowHeight="8400" tabRatio="600" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="21000" windowHeight="8400" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="PAGE" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="LOCATOR" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="TEST_CASES" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="TEST_STEPS" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="TEST_DATA" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="ACTION" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="TEST_CASE" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="OBJECT_REPOSITORY" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
-  <definedNames>
-    <definedName name="actions">ACTION!$A$1:$A$20</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -25,7 +22,7 @@
     <numFmt numFmtId="164" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="165" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -36,7 +33,14 @@
     <font>
       <name val="Calibri"/>
       <charset val="134"/>
-      <color theme="10"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF0000FF"/>
       <sz val="11"/>
       <u val="single"/>
       <scheme val="minor"/>
@@ -178,18 +182,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="33">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.249977111117893"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -486,157 +484,154 @@
     </border>
   </borders>
   <cellStyleXfs count="49">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="4" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="6" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="18" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="30" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="6"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1049,35 +1044,57 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="2"/>
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="4"/>
   <cols>
-    <col width="14.7222222222222" customWidth="1" min="1" max="1"/>
-    <col width="16.0925925925926" customWidth="1" min="2" max="2"/>
-    <col width="53.4537037037037" customWidth="1" min="3" max="3"/>
+    <col width="13.5555555555556" customWidth="1" min="1" max="1"/>
+    <col width="14.8888888888889" customWidth="1" min="2" max="2"/>
+    <col width="24.2222222222222" customWidth="1" min="3" max="3"/>
+    <col width="8.33333333333333" customWidth="1" min="4" max="4"/>
+    <col width="10.1111111111111" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>page_id</t>
+          <t>TestCaseID</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>page_name</t>
+          <t>Module</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>url</t>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Duration</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>login</t>
+          <t>TC_LOGIN_01</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1085,34 +1102,145 @@
           <t>Login</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>https://qa-automation-practice.netlify.app/auth_ecommerce</t>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Login success</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>8.78s</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>home_page</t>
+          <t>TC_EMR_01</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>Medical Record</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>/home</t>
+          <t>View patient profile</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>10.01s</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TC_AI_01</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Diagnosis AI</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Analyze disease</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>10.04s</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TC_REM_01</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Reminder</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Create medicine reminder</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>10.02s</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" display="https://qa-automation-practice.netlify.app/auth_ecommerce" r:id="rId1"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -1122,180 +1250,719 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="5"/>
+  <dimension ref="A1:I17"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col width="17.8148148148148" customWidth="1" min="1" max="1"/>
-    <col width="10.3611111111111" customWidth="1" min="2" max="2"/>
-    <col width="19.8888888888889" customWidth="1" min="3" max="3"/>
-    <col width="15.5462962962963" customWidth="1" min="4" max="4"/>
-    <col width="20.3611111111111" customWidth="1" min="5" max="5"/>
+    <col width="21.1111111111111" customWidth="1" min="4" max="4"/>
+    <col width="15.6666666666667" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>element_id</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>page_id</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>element_name</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>element_type</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>locator_value</t>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>TestCaseID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>StepNo</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>TargetElement</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>TestDataKey</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>ExpectedResult</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>ActualResult</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Duration</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>txt_email</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>login</t>
-        </is>
+          <t>TC_LOGIN_01</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Email textbox</t>
+          <t>navigate</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>input</t>
+          <t>url_login</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>#email</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Login page displayed</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Navigated to https://qa-automation-practice.netlify.app/auth_ecommerce</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>8.34s</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>txt_password</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>login</t>
-        </is>
+          <t>TC_LOGIN_01</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Password textbox</t>
+          <t>input</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>input</t>
+          <t>txt_username</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>#password</t>
+          <t>doctor_user</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Username entered</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Input 'admin@admin.com' into txt_username</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>0.15s</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>btn_login</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>login</t>
-        </is>
+          <t>TC_LOGIN_01</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Login button</t>
+          <t>input</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>button</t>
+          <t>txt_password</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>button[type='submit']</t>
+          <t>doctor_pass</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Password entered</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Input 'admin123' into txt_password</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>0.13s</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>msg_error</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>login</t>
-        </is>
+          <t>TC_LOGIN_01</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Error message</t>
+          <t>click</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>btn_login</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>#message</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Dashboard displayed</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Clicked btn_login</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>0.15s</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>lbl_shopping_cart</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
+          <t>TC_EMR_01</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Shopping cart header</t>
+          <t>click</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>menu_medical_record</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>h2.section-header</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Medical record list shown</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error: Message: 
+Stacktrace:
+	chromedriver!GetHandleVerifier [0x6b7123+10a23]
+	chromedriver!GetHandleVerifier [0x6b7254+10b54]
+	chromedriver!(No symbol) [0x4d1e90]
+	chromedriver!(No symbol) [0x51b28a]
+	chromedriver!(No symbol) [0x51b52b]
+	chromedriver!(No symbol) [0x55d062]
+	chromedriver!(No symbol) [0x53d7d4]
+	chromedriver!(No symbol) [0x55a936]
+	chromedriver!(No symbol) [0x53d526]
+	chromedriver!(No symbol) [0x5108f9]
+	chromedriver!(No symbol) [0x5116b4]
+	chromedriver!GetHandleVerifier [0x951ac4+2ab3c4]
+	chromedriver!GetHandleVerifier [0x94d0ed+2a69ed]
+	chromedriver!GetHandleVerifier [0x96e4f5+2c7df5]
+	chromedriver!GetHandleVerifier [0x6d1128+2aa28]
+	chromedriver!GetHandleVerifier [0x6d8bbd+324bd]
+	chromedriver!GetHandleVerifier [0x6bfb28+19428]
+	chromedriver!GetHandleVerifier [0x6bfcd5+195d5]
+	chromedriver!GetHandleVerifier [0x6a91cf+2acf]
+	KERNEL32!BaseThreadInitThunk [0x75cc5d49+19]
+	ntdll!RtlInitializeExceptionChain [0x775dd83b+6b]
+	ntdll!RtlGetAppContainerNamedObjectPath [0x775dd7c1+231]
+</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>10.01s</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TC_EMR_01</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>patient_row</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>patient_id_001</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Patient profile opened</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TC_EMR_01</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>verify</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>lbl_patient_name</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>patient_name</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Correct patient info shown</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TC_AI_01</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>btn_ai_analyze</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>AI processing started</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error: Message: 
+Stacktrace:
+	chromedriver!GetHandleVerifier [0x6b7123+10a23]
+	chromedriver!GetHandleVerifier [0x6b7254+10b54]
+	chromedriver!(No symbol) [0x4d1e90]
+	chromedriver!(No symbol) [0x51b28a]
+	chromedriver!(No symbol) [0x51b52b]
+	chromedriver!(No symbol) [0x55d062]
+	chromedriver!(No symbol) [0x53d7d4]
+	chromedriver!(No symbol) [0x55a936]
+	chromedriver!(No symbol) [0x53d526]
+	chromedriver!(No symbol) [0x5108f9]
+	chromedriver!(No symbol) [0x5116b4]
+	chromedriver!GetHandleVerifier [0x951ac4+2ab3c4]
+	chromedriver!GetHandleVerifier [0x94d0ed+2a69ed]
+	chromedriver!GetHandleVerifier [0x96e4f5+2c7df5]
+	chromedriver!GetHandleVerifier [0x6d1128+2aa28]
+	chromedriver!GetHandleVerifier [0x6d8bbd+324bd]
+	chromedriver!GetHandleVerifier [0x6bfb28+19428]
+	chromedriver!GetHandleVerifier [0x6bfcd5+195d5]
+	chromedriver!GetHandleVerifier [0x6a91cf+2acf]
+	KERNEL32!BaseThreadInitThunk [0x75cc5d49+19]
+	ntdll!RtlInitializeExceptionChain [0x775dd83b+6b]
+	ntdll!RtlGetAppContainerNamedObjectPath [0x775dd7c1+231]
+</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>10.04s</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TC_AI_01</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>wait</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ai_loading</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>AI loading displayed</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TC_AI_01</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>3</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>verify</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>lbl_diagnosis</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>diagnosis_text</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Diagnosis result displayed</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TC_AI_01</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>verify</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>lbl_confidence</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>confidence_rate</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Confidence shown</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TC_REM_01</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>btn_create_reminder</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Reminder form opened</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error: Message: 
+Stacktrace:
+	chromedriver!GetHandleVerifier [0x6b7123+10a23]
+	chromedriver!GetHandleVerifier [0x6b7254+10b54]
+	chromedriver!(No symbol) [0x4d1e90]
+	chromedriver!(No symbol) [0x51b28a]
+	chromedriver!(No symbol) [0x51b52b]
+	chromedriver!(No symbol) [0x55d062]
+	chromedriver!(No symbol) [0x53d7d4]
+	chromedriver!(No symbol) [0x55a936]
+	chromedriver!(No symbol) [0x53d526]
+	chromedriver!(No symbol) [0x5108f9]
+	chromedriver!(No symbol) [0x5116b4]
+	chromedriver!GetHandleVerifier [0x951ac4+2ab3c4]
+	chromedriver!GetHandleVerifier [0x94d0ed+2a69ed]
+	chromedriver!GetHandleVerifier [0x96e4f5+2c7df5]
+	chromedriver!GetHandleVerifier [0x6d1128+2aa28]
+	chromedriver!GetHandleVerifier [0x6d8bbd+324bd]
+	chromedriver!GetHandleVerifier [0x6bfb28+19428]
+	chromedriver!GetHandleVerifier [0x6bfcd5+195d5]
+	chromedriver!GetHandleVerifier [0x6a91cf+2acf]
+	KERNEL32!BaseThreadInitThunk [0x75cc5d49+19]
+	ntdll!RtlInitializeExceptionChain [0x775dd83b+6b]
+	ntdll!RtlGetAppContainerNamedObjectPath [0x775dd7c1+231]
+</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>10.02s</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TC_REM_01</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>txt_medicine_name</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>medicine_name</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Medicine name entered</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>TC_REM_01</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>select</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>dropdown_frequency</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>frequency_daily</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Frequency selected</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TC_REM_01</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>btn_save</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Reminder created successfully</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>TC_REM_01</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>5</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>verify</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>lbl_reminder_status</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>reminder_active</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Reminder active</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -1305,32 +1972,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="5"/>
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col width="18.3611111111111" customWidth="1" min="1" max="1"/>
-    <col width="29.1759259259259" customWidth="1" min="2" max="2"/>
+    <col width="15.6666666666667" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>data_key</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>value</t>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>DataKey</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Value</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>valid_email</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
+          <t>doctor_user</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>admin@admin.com</t>
         </is>
@@ -1339,7 +2005,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>valid_password</t>
+          <t>doctor_pass</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1351,43 +2017,89 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>invalid_password</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>123456</v>
+          <t>patient_id_001</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>P0001</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>error_text</t>
+          <t>patient_name</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Bad credentials! Please try again! Make sure that you've registered.</t>
+          <t>Nguyen Van A</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>shopping_cart_text</t>
+          <t>diagnosis_text</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>SHOPPING CART</t>
+          <t>Risk of Hypertension</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>confidence_rate</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>&gt;80%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>medicine_name</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Paracetamol</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>frequency_daily</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Daily</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>reminder_active</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" display="admin@admin.com" r:id="rId1"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" paperSize="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -1397,321 +2109,304 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="4"/>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col width="16.6296296296296" customWidth="1" min="1" max="1"/>
-    <col width="21.2685185185185" customWidth="1" min="2" max="2"/>
-    <col width="16.5462962962963" customWidth="1" min="3" max="3"/>
-    <col width="11.9074074074074" customWidth="1" min="4" max="4"/>
-    <col width="15.4537037037037" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="21.1111111111111" customWidth="1" min="1" max="1"/>
+    <col width="12.1111111111111" customWidth="1" min="2" max="2"/>
+    <col width="56.8888888888889" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>action</t>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ElementKey</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>LocatorType</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>LocatorValue</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>navigate</t>
+          <t>txt_username</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>email</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>input</t>
+          <t>txt_password</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>password</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>input</t>
+          <t>btn_login</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>submitLoginBtn</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>check</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G11"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4"/>
-  <cols>
-    <col width="14.8148148148148" customWidth="1" min="1" max="1"/>
-    <col width="29.3611111111111" customWidth="1" min="2" max="2"/>
-    <col width="12.3611111111111" customWidth="1" min="5" max="5"/>
-    <col width="16.7777777777778" customWidth="1" min="6" max="6"/>
-    <col width="18.2222222222222" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>tc_id</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>type</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>step</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>action</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>target</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>data</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>TC_LOGIN_001</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Login success</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>happy</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>navigate</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>login_page</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="D3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>input</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>txt_email</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>valid_email</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="D4" t="n">
-        <v>3</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>input</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>txt_password</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>valid_password</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="D5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>click</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>btn_login</t>
+          <t>menu_medical_record</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>xpath</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>//a[text()='Medical Records']</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="D6" t="n">
-        <v>5</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>check</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>lbl_shopping_cart</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>shopping_cart_text</t>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>btn_ai_analyze</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>btnAnalyze</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TC_LOGIN_002</t>
+          <t>lbl_diagnosis</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Login wrong password</t>
+          <t>id</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>negative</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>navigate</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>login_page</t>
+          <t>diagnosisResult</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="D8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>input</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>txt_email</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>valid_email</t>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>btn_create_reminder</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>createReminder</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="D9" t="n">
-        <v>3</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>input</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>txt_password</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>invalid_password</t>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>url_login</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://qa-automation-practice.netlify.app/auth_ecommerce</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="D10" t="n">
-        <v>4</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>click</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>btn_login</t>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>patient_row</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>patient_001</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="D11" t="n">
-        <v>5</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>check</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>lbl_error</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>error_text</t>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>lbl_patient_name</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>patientName</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ai_loading</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>loadingSpinner</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>lbl_confidence</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>confidenceScore</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>txt_medicine_name</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>medicineInput</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>dropdown_frequency</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>freqSelect</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>btn_save</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>saveBtn</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>lbl_reminder_status</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>reminderStatus</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>